<commit_message>
Sensor params from the team sensor slides: GPS-L10 10 Hz, VN-100 IMU noise
GPS rate 20 -> 10 Hz (MoTeC GPS-L10, one fitted — slide 79). IMU identified
as a VectorNav VN-100 (slide 75); gyro/accel noise and gyro bias set to its
datasheet figures from memory, tagged VERIFY. Table and sheet regenerated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/datasheets/FSAE-Sim Parameters.xlsx
+++ b/docs/datasheets/FSAE-Sim Parameters.xlsx
@@ -11268,12 +11268,12 @@
       </c>
       <c r="D225" s="3" t="inlineStr">
         <is>
-          <t>Yaw-gyro 1-sigma noise.</t>
+          <t>Yaw-gyro 1-sigma noise per 100 Hz sample. The car's IMU is a VN-100 (team sensor slide 75).</t>
         </is>
       </c>
       <c r="E225" s="4" t="inlineStr">
         <is>
-          <t>0.005236</t>
+          <t>0.0004363</t>
         </is>
       </c>
       <c r="F225" s="3" t="inlineStr">
@@ -11283,17 +11283,17 @@
       </c>
       <c r="G225" s="5" t="inlineStr">
         <is>
-          <t>PLACEHOLDER — IMU spec</t>
+          <t>PLACEHOLDER — VectorNav VN-100 datasheet value from memory (0.0035 deg/s/sqrt(Hz) x sqrt(50 Hz)); VERIFY against the sheet</t>
         </is>
       </c>
       <c r="H225" s="3" t="inlineStr">
         <is>
-          <t>IMU datasheet numbers</t>
+          <t>Confirm the VN-100 noise density on its datasheet</t>
         </is>
       </c>
       <c r="I225" s="3" t="inlineStr">
         <is>
-          <t>Chosen IMU's spec sheet</t>
+          <t>VN-100 datasheet: noise density x sqrt(VCU bandwidth)</t>
         </is>
       </c>
       <c r="J225" s="3" t="inlineStr">
@@ -11320,12 +11320,12 @@
       </c>
       <c r="D226" s="3" t="inlineStr">
         <is>
-          <t>Constant yaw-gyro zero offset.</t>
+          <t>Constant yaw-gyro zero offset left after the VN-100's own calibration.</t>
         </is>
       </c>
       <c r="E226" s="4" t="inlineStr">
         <is>
-          <t>0.001745</t>
+          <t>5.236e-05</t>
         </is>
       </c>
       <c r="F226" s="3" t="inlineStr">
@@ -11335,17 +11335,17 @@
       </c>
       <c r="G226" s="5" t="inlineStr">
         <is>
-          <t>PLACEHOLDER — uncalibrated bias</t>
+          <t>PLACEHOLDER — VN-100 in-run bias stability (~10 deg/hr) from memory; VERIFY, then calibrate on the car</t>
         </is>
       </c>
       <c r="H226" s="3" t="inlineStr">
         <is>
-          <t>IMU datasheet numbers</t>
+          <t>Stationary log on the car</t>
         </is>
       </c>
       <c r="I226" s="3" t="inlineStr">
         <is>
-          <t>Chosen IMU's spec sheet, then a stationary calibration on the car</t>
+          <t>VN-100 datasheet bias stability, then a stationary calibration on the car</t>
         </is>
       </c>
       <c r="J226" s="3" t="inlineStr">
@@ -11424,12 +11424,12 @@
       </c>
       <c r="D228" s="3" t="inlineStr">
         <is>
-          <t>Accelerometer 1-sigma noise (ax, ay channels).</t>
+          <t>Accelerometer 1-sigma noise per 100 Hz sample (ax, ay channels). The car's IMU is a VN-100 (team sensor slide 75).</t>
         </is>
       </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="F228" s="3" t="inlineStr">
@@ -11439,17 +11439,17 @@
       </c>
       <c r="G228" s="5" t="inlineStr">
         <is>
-          <t>PLACEHOLDER — IMU spec</t>
+          <t>PLACEHOLDER — VN-100 datasheet value from memory (0.14 mg/sqrt(Hz) x sqrt(50 Hz)); VERIFY</t>
         </is>
       </c>
       <c r="H228" s="3" t="inlineStr">
         <is>
-          <t>IMU datasheet</t>
+          <t>Confirm the VN-100 accel noise density on its datasheet</t>
         </is>
       </c>
       <c r="I228" s="3" t="inlineStr">
         <is>
-          <t>Spec sheet</t>
+          <t>VN-100 datasheet: noise density x sqrt(VCU bandwidth)</t>
         </is>
       </c>
       <c r="J228" s="3" t="inlineStr">
@@ -11691,12 +11691,12 @@
       </c>
       <c r="D234" s="3" t="inlineStr">
         <is>
-          <t>How often each receiver produces a new speed.</t>
-        </is>
-      </c>
-      <c r="E234" s="4" t="inlineStr">
-        <is>
-          <t>20</t>
+          <t>How often each receiver produces a new speed. SR-17 carries ONE GPS-L10; the model's second receiver (and its bias state) is the DOF doc's provision, not fitted hardware.</t>
+        </is>
+      </c>
+      <c r="E234" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="F234" s="3" t="inlineStr">
@@ -11704,19 +11704,19 @@
           <t>Hz</t>
         </is>
       </c>
-      <c r="G234" s="5" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER — receiver datasheet</t>
+      <c r="G234" s="7" t="inlineStr">
+        <is>
+          <t>CURRENT CAR (MoTeC GPS-L10, team sensor slide 79)</t>
         </is>
       </c>
       <c r="H234" s="3" t="inlineStr">
         <is>
-          <t>Receiver datasheet / configured rate</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I234" s="3" t="inlineStr">
         <is>
-          <t>Datasheet</t>
+          <t>Sensor slide 79 (MoTeC GPS-L10 datasheet: 10 Hz)</t>
         </is>
       </c>
       <c r="J234" s="3" t="inlineStr">

</xml_diff>